<commit_message>
Ship the RTS-96 case files the paper used
Both files now match the inputs behind the paper's RTS-96 results:
IC6 controls reactive power (CQ) instead of the AC voltage at bus 215,
which a generator already holds; the lower frequency bound is 0.975 pu;
the droop case carries the corrected IC active-power set-points; and DC
loads use the ZIP columns (Z_p, I_p, P_p).
</commit_message>
<xml_diff>
--- a/grids/rts96_scenario1_constant_vdc.xlsx
+++ b/grids/rts96_scenario1_constant_vdc.xlsx
@@ -2030,7 +2030,7 @@
         <v>6</v>
       </c>
       <c r="C7">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D7">
         <v>0</v>
@@ -2398,7 +2398,7 @@
         <v>1</v>
       </c>
       <c r="D2">
-        <v>0.97499999999999998</v>
+        <v>0.975</v>
       </c>
       <c r="E2">
         <v>1.02</v>
@@ -5150,38 +5150,50 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="4.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.1640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="4" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.1640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:8">
       <c r="A1" t="s">
         <v>1</v>
       </c>
-      <c r="B1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Z_p</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>I_p</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>P_p</t>
+        </is>
+      </c>
+      <c r="E1" t="s">
         <v>12</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>14</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>19</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:8">
       <c r="A2">
         <v>1</v>
       </c>
@@ -5189,19 +5201,25 @@
         <v>0</v>
       </c>
       <c r="C2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2">
         <v>150000</v>
       </c>
-      <c r="E2">
+      <c r="G2">
         <v>0.9</v>
       </c>
-      <c r="F2">
+      <c r="H2">
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:8">
       <c r="A3">
         <v>2</v>
       </c>
@@ -5209,19 +5227,25 @@
         <v>0</v>
       </c>
       <c r="C3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3">
         <v>150000</v>
       </c>
-      <c r="E3">
+      <c r="G3">
         <v>0.9</v>
       </c>
-      <c r="F3">
+      <c r="H3">
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:8">
       <c r="A4">
         <v>3</v>
       </c>
@@ -5229,19 +5253,25 @@
         <v>0</v>
       </c>
       <c r="C4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="F4">
         <v>150000</v>
       </c>
-      <c r="E4">
+      <c r="G4">
         <v>0.9</v>
       </c>
-      <c r="F4">
+      <c r="H4">
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:8">
       <c r="A5">
         <v>4</v>
       </c>
@@ -5249,19 +5279,25 @@
         <v>0</v>
       </c>
       <c r="C5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="F5">
         <v>300000</v>
       </c>
-      <c r="E5">
+      <c r="G5">
         <v>0.9</v>
       </c>
-      <c r="F5">
+      <c r="H5">
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:8">
       <c r="A6">
         <v>5</v>
       </c>
@@ -5269,19 +5305,25 @@
         <v>0</v>
       </c>
       <c r="C6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="F6">
         <v>300000</v>
       </c>
-      <c r="E6">
+      <c r="G6">
         <v>0.9</v>
       </c>
-      <c r="F6">
+      <c r="H6">
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:8">
       <c r="A7">
         <v>6</v>
       </c>
@@ -5289,19 +5331,25 @@
         <v>0</v>
       </c>
       <c r="C7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="F7">
         <v>300000</v>
       </c>
-      <c r="E7">
+      <c r="G7">
         <v>0.9</v>
       </c>
-      <c r="F7">
+      <c r="H7">
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:8">
       <c r="A8">
         <v>7</v>
       </c>
@@ -5309,15 +5357,21 @@
         <v>0</v>
       </c>
       <c r="C8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+      <c r="F8">
         <v>300000</v>
       </c>
-      <c r="E8">
+      <c r="G8">
         <v>0.9</v>
       </c>
-      <c r="F8">
+      <c r="H8">
         <v>1.1000000000000001</v>
       </c>
     </row>

</xml_diff>